<commit_message>
review code for ai and performance optimizer
</commit_message>
<xml_diff>
--- a/sections_config.xlsx
+++ b/sections_config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13a0fd42d83c08bf/Documents/Cursos/ILLINOIS/IE_421_High_Frequency_Trading/LinuxVM/project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13a0fd42d83c08bf/Documents/Cursos/ILLINOIS/IE_421_High_Frequency_Trading/LinuxVM/LLM_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2BC6806-065A-0848-B249-98B965329BD7}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12DE9B4A-A904-2B4A-AE77-C440D208F5B1}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="1660" windowWidth="27240" windowHeight="16160" xr2:uid="{D840E18A-208A-1543-8781-3BD2E5582C66}"/>
   </bookViews>
@@ -531,10 +531,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1761,7 +1757,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -1778,7 +1774,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>114</v>
       </c>
@@ -1790,6 +1786,9 @@
       </c>
       <c r="D53" t="s">
         <v>84</v>
+      </c>
+      <c r="F53">
+        <v>15</v>
       </c>
       <c r="H53" t="s">
         <v>137</v>
@@ -1808,6 +1807,12 @@
       <c r="D54" t="s">
         <v>84</v>
       </c>
+      <c r="E54">
+        <v>30</v>
+      </c>
+      <c r="F54">
+        <v>100</v>
+      </c>
       <c r="H54" t="s">
         <v>139</v>
       </c>
@@ -1825,6 +1830,9 @@
       <c r="D55" t="s">
         <v>84</v>
       </c>
+      <c r="F55">
+        <v>5</v>
+      </c>
       <c r="H55" t="s">
         <v>139</v>
       </c>
@@ -1842,6 +1850,9 @@
       <c r="D56" t="s">
         <v>84</v>
       </c>
+      <c r="F56">
+        <v>10</v>
+      </c>
       <c r="H56" t="s">
         <v>139</v>
       </c>
@@ -1862,9 +1873,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H57" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}">
-    <filterColumn colId="7">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Storage"/>
+        <filter val="vda Average wait time"/>
+        <filter val="vda I/O Statistics"/>
+        <filter val="vda Read wait time"/>
+        <filter val="vda Utilization percentage"/>
+        <filter val="vda Write wait time"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
improved code + Added Universal AI config
</commit_message>
<xml_diff>
--- a/sections_config.xlsx
+++ b/sections_config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13a0fd42d83c08bf/Documents/Cursos/ILLINOIS/IE_421_High_Frequency_Trading/LinuxVM/LLM_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12DE9B4A-A904-2B4A-AE77-C440D208F5B1}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0EB680B-A3DB-D94B-84D9-24E9883CAB39}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="1660" windowWidth="27240" windowHeight="16160" xr2:uid="{D840E18A-208A-1543-8781-3BD2E5582C66}"/>
   </bookViews>
@@ -531,6 +531,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -850,7 +854,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -886,7 +889,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>50</v>
       </c>
@@ -903,7 +906,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -920,7 +923,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -937,7 +940,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -954,7 +957,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -971,7 +974,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
@@ -988,7 +991,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1005,7 +1008,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1022,7 +1025,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -1039,7 +1042,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -1056,7 +1059,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -1090,7 +1093,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -1124,7 +1127,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
@@ -1141,7 +1144,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -1158,7 +1161,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>56</v>
       </c>
@@ -1175,7 +1178,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>56</v>
       </c>
@@ -1192,7 +1195,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>61</v>
       </c>
@@ -1209,7 +1212,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>66</v>
       </c>
@@ -1243,7 +1246,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>69</v>
       </c>
@@ -1260,7 +1263,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>69</v>
       </c>
@@ -1277,7 +1280,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>74</v>
       </c>
@@ -1294,7 +1297,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>77</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>77</v>
       </c>
@@ -1328,7 +1331,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>19</v>
       </c>
@@ -1345,7 +1348,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>19</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>19</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -1396,7 +1399,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>19</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>19</v>
       </c>
@@ -1430,7 +1433,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
@@ -1447,7 +1450,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>19</v>
       </c>
@@ -1470,7 +1473,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>19</v>
       </c>
@@ -1493,7 +1496,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>19</v>
       </c>
@@ -1516,7 +1519,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>19</v>
       </c>
@@ -1536,7 +1539,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>19</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>19</v>
       </c>
@@ -1570,7 +1573,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>19</v>
       </c>
@@ -1587,7 +1590,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
@@ -1604,7 +1607,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>19</v>
       </c>
@@ -1621,7 +1624,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1638,7 +1641,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -1655,7 +1658,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -1672,7 +1675,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -1689,7 +1692,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>19</v>
       </c>
@@ -1706,7 +1709,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -1723,7 +1726,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>27</v>
       </c>
@@ -1740,7 +1743,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>27</v>
       </c>
@@ -1857,7 +1860,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -1872,17 +1875,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H57" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="vda Average wait time"/>
-        <filter val="vda I/O Statistics"/>
-        <filter val="vda Read wait time"/>
-        <filter val="vda Utilization percentage"/>
-        <filter val="vda Write wait time"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H57" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BIOS + Application Code
</commit_message>
<xml_diff>
--- a/sections_config.xlsx
+++ b/sections_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13a0fd42d83c08bf/Documents/Cursos/ILLINOIS/IE_421_High_Frequency_Trading/LinuxVM/LLM_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0EB680B-A3DB-D94B-84D9-24E9883CAB39}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{17DEADED-3F36-7A45-9954-13B779C8B78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11E793DF-5168-5A4B-B2E8-FCF94D3BAC2D}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="1660" windowWidth="27240" windowHeight="16160" xr2:uid="{D840E18A-208A-1543-8781-3BD2E5582C66}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Sections" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sections!$A$1:$H$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sections!$A$1:$H$56</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="154">
   <si>
     <t>Section_Title</t>
   </si>
@@ -462,6 +462,45 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>BIOS &amp; Firmware</t>
+  </si>
+  <si>
+    <t>BIOS Version &amp; Date</t>
+  </si>
+  <si>
+    <t>dmidecode -t 0 2&gt;/dev/null | cat</t>
+  </si>
+  <si>
+    <t>Motherboard &amp; Chipset</t>
+  </si>
+  <si>
+    <t>dmidecode -t 2 2&gt;/dev/null | cat</t>
+  </si>
+  <si>
+    <t>CPU Power States</t>
+  </si>
+  <si>
+    <t>cpupower frequency-info 2&gt;/dev/null | cat</t>
+  </si>
+  <si>
+    <t>Idle States (C-states)</t>
+  </si>
+  <si>
+    <t>cpupower idle-info 2&gt;/dev/null | cat</t>
+  </si>
+  <si>
+    <t>PCIe Power Management (ASPM)</t>
+  </si>
+  <si>
+    <t>lspci -vvv | grep -E "ASPM|L1|L2|Power Management" 2&gt;/dev/null</t>
+  </si>
+  <si>
+    <t>CPU Flags &amp; Mitigations</t>
+  </si>
+  <si>
+    <t>cat /proc/cpuinfo | grep -E "flags|bugs" | head -10</t>
   </si>
 </sst>
 </file>
@@ -854,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.5" bestFit="1" customWidth="1"/>
@@ -1861,21 +1900,123 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="A57" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>125</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B63" t="s">
         <v>130</v>
       </c>
-      <c r="D57" t="s">
-        <v>53</v>
-      </c>
-      <c r="H57" t="s">
+      <c r="D63" t="s">
+        <v>53</v>
+      </c>
+      <c r="H63" t="s">
         <v>140</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H57" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}"/>
+  <autoFilter ref="A1:H56" xr:uid="{F7F98F07-8A77-3547-A6A2-1E1EBA77126D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>